<commit_message>
Dark green theme, nutrition info, Telegram link
- Deep green background with saffron accent
- Detail panel shows calories, protein, fat and carbs per portion (rough estimates from new menu.xlsx columns)
- Floating «Наш Telegram» button and a Telegram card at the end of the menu (t.me/otziv_chay)
</commit_message>
<xml_diff>
--- a/menu.xlsx
+++ b/menu.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E132"/>
+  <dimension ref="A1:I132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -431,6 +431,10 @@
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -459,6 +463,26 @@
           <t>Фото</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Калории</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Белки</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Жиры</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Углеводы</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -484,6 +508,18 @@
           <t>product_1778499752830_7fdac0d85fd1.webp</t>
         </is>
       </c>
+      <c r="F2" t="n">
+        <v>278</v>
+      </c>
+      <c r="G2" t="n">
+        <v>19</v>
+      </c>
+      <c r="H2" t="n">
+        <v>22</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -509,6 +545,18 @@
           <t>product_1780238620613_aca1e752351e.webp</t>
         </is>
       </c>
+      <c r="F3" t="n">
+        <v>298</v>
+      </c>
+      <c r="G3" t="n">
+        <v>19</v>
+      </c>
+      <c r="H3" t="n">
+        <v>22</v>
+      </c>
+      <c r="I3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -534,6 +582,18 @@
           <t>product_1778788909754_dcc49604d37c.webp</t>
         </is>
       </c>
+      <c r="F4" t="n">
+        <v>328</v>
+      </c>
+      <c r="G4" t="n">
+        <v>20</v>
+      </c>
+      <c r="H4" t="n">
+        <v>24</v>
+      </c>
+      <c r="I4" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -559,6 +619,18 @@
           <t>product_1780238659096_72d3ced28b94.webp</t>
         </is>
       </c>
+      <c r="F5" t="n">
+        <v>418</v>
+      </c>
+      <c r="G5" t="n">
+        <v>25</v>
+      </c>
+      <c r="H5" t="n">
+        <v>34</v>
+      </c>
+      <c r="I5" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -584,6 +656,18 @@
           <t>product_1778336306724_09d809d12a06.webp</t>
         </is>
       </c>
+      <c r="F6" t="n">
+        <v>294</v>
+      </c>
+      <c r="G6" t="n">
+        <v>16</v>
+      </c>
+      <c r="H6" t="n">
+        <v>22</v>
+      </c>
+      <c r="I6" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -609,6 +693,18 @@
           <t>product_1778336450597_568824ff5179.webp</t>
         </is>
       </c>
+      <c r="F7" t="n">
+        <v>234</v>
+      </c>
+      <c r="G7" t="n">
+        <v>10</v>
+      </c>
+      <c r="H7" t="n">
+        <v>18</v>
+      </c>
+      <c r="I7" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -634,6 +730,18 @@
           <t>product_1778791161570_899c5ebb81ff.webp</t>
         </is>
       </c>
+      <c r="F8" t="n">
+        <v>312</v>
+      </c>
+      <c r="G8" t="n">
+        <v>16</v>
+      </c>
+      <c r="H8" t="n">
+        <v>24</v>
+      </c>
+      <c r="I8" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -659,6 +767,18 @@
           <t>product_1778791224697_82046e277e77.webp</t>
         </is>
       </c>
+      <c r="F9" t="n">
+        <v>244</v>
+      </c>
+      <c r="G9" t="n">
+        <v>5</v>
+      </c>
+      <c r="H9" t="n">
+        <v>16</v>
+      </c>
+      <c r="I9" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -684,6 +804,18 @@
           <t>product_1778338170859_73f84b2653f1.webp</t>
         </is>
       </c>
+      <c r="F10" t="n">
+        <v>304</v>
+      </c>
+      <c r="G10" t="n">
+        <v>16</v>
+      </c>
+      <c r="H10" t="n">
+        <v>24</v>
+      </c>
+      <c r="I10" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -709,6 +841,18 @@
           <t>product_1778338214857_66a9bf0fe63f.webp</t>
         </is>
       </c>
+      <c r="F11" t="n">
+        <v>350</v>
+      </c>
+      <c r="G11" t="n">
+        <v>24</v>
+      </c>
+      <c r="H11" t="n">
+        <v>22</v>
+      </c>
+      <c r="I11" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -734,6 +878,18 @@
           <t>product_1778791590329_87a69efebfa5.webp</t>
         </is>
       </c>
+      <c r="F12" t="n">
+        <v>330</v>
+      </c>
+      <c r="G12" t="n">
+        <v>16</v>
+      </c>
+      <c r="H12" t="n">
+        <v>26</v>
+      </c>
+      <c r="I12" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -759,6 +915,18 @@
           <t>product_1778791691448_c2f843c30b81.webp</t>
         </is>
       </c>
+      <c r="F13" t="n">
+        <v>242</v>
+      </c>
+      <c r="G13" t="n">
+        <v>15</v>
+      </c>
+      <c r="H13" t="n">
+        <v>14</v>
+      </c>
+      <c r="I13" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -784,6 +952,18 @@
           <t>product_1778340272766_05294196e0a5.webp</t>
         </is>
       </c>
+      <c r="F14" t="n">
+        <v>294</v>
+      </c>
+      <c r="G14" t="n">
+        <v>16</v>
+      </c>
+      <c r="H14" t="n">
+        <v>22</v>
+      </c>
+      <c r="I14" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -809,6 +989,18 @@
           <t>product_1778340354580_2cbdb7edea11.webp</t>
         </is>
       </c>
+      <c r="F15" t="n">
+        <v>302</v>
+      </c>
+      <c r="G15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H15" t="n">
+        <v>22</v>
+      </c>
+      <c r="I15" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -834,6 +1026,18 @@
           <t>product_1778792774726_cd1fff651a3f.webp</t>
         </is>
       </c>
+      <c r="F16" t="n">
+        <v>398</v>
+      </c>
+      <c r="G16" t="n">
+        <v>18</v>
+      </c>
+      <c r="H16" t="n">
+        <v>30</v>
+      </c>
+      <c r="I16" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -859,6 +1063,18 @@
           <t>product_1778340507491_b449f3a7578f.webp</t>
         </is>
       </c>
+      <c r="F17" t="n">
+        <v>346</v>
+      </c>
+      <c r="G17" t="n">
+        <v>12</v>
+      </c>
+      <c r="H17" t="n">
+        <v>26</v>
+      </c>
+      <c r="I17" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -884,6 +1100,18 @@
           <t>product_1778340622299_d0880974280d.webp</t>
         </is>
       </c>
+      <c r="F18" t="n">
+        <v>182</v>
+      </c>
+      <c r="G18" t="n">
+        <v>3</v>
+      </c>
+      <c r="H18" t="n">
+        <v>10</v>
+      </c>
+      <c r="I18" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -909,6 +1137,18 @@
           <t>product_1778340699538_9b1f7d1d7c94.webp</t>
         </is>
       </c>
+      <c r="F19" t="n">
+        <v>252</v>
+      </c>
+      <c r="G19" t="n">
+        <v>8</v>
+      </c>
+      <c r="H19" t="n">
+        <v>20</v>
+      </c>
+      <c r="I19" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -929,6 +1169,18 @@
           <t>Помидоры, огурцы, красный лук, грецкий орех, кинза, базилик, растительное масло</t>
         </is>
       </c>
+      <c r="F20" t="n">
+        <v>244</v>
+      </c>
+      <c r="G20" t="n">
+        <v>6</v>
+      </c>
+      <c r="H20" t="n">
+        <v>20</v>
+      </c>
+      <c r="I20" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -954,6 +1206,18 @@
           <t>product_1778794108968_bf32dfc6bb16.webp</t>
         </is>
       </c>
+      <c r="F21" t="n">
+        <v>93</v>
+      </c>
+      <c r="G21" t="n">
+        <v>2</v>
+      </c>
+      <c r="H21" t="n">
+        <v>5</v>
+      </c>
+      <c r="I21" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -979,6 +1243,18 @@
           <t>product_1778794320866_9c6311fc066e.webp</t>
         </is>
       </c>
+      <c r="F22" t="n">
+        <v>138</v>
+      </c>
+      <c r="G22" t="n">
+        <v>3</v>
+      </c>
+      <c r="H22" t="n">
+        <v>10</v>
+      </c>
+      <c r="I22" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1004,6 +1280,18 @@
           <t>product_1778794382827_1e9c6ef6714a.webp</t>
         </is>
       </c>
+      <c r="F23" t="n">
+        <v>214</v>
+      </c>
+      <c r="G23" t="n">
+        <v>14</v>
+      </c>
+      <c r="H23" t="n">
+        <v>14</v>
+      </c>
+      <c r="I23" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1024,6 +1312,18 @@
           <t>Капуста, огурцы, морковь, зелень, лимонная заправка</t>
         </is>
       </c>
+      <c r="F24" t="n">
+        <v>120</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" t="n">
+        <v>8</v>
+      </c>
+      <c r="I24" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1044,6 +1344,18 @@
           <t>Отварная свёкла, чеснок, грецкий орех, майонез</t>
         </is>
       </c>
+      <c r="F25" t="n">
+        <v>278</v>
+      </c>
+      <c r="G25" t="n">
+        <v>4</v>
+      </c>
+      <c r="H25" t="n">
+        <v>22</v>
+      </c>
+      <c r="I25" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1064,6 +1376,18 @@
           <t>Сельдь, свёкла, картофель, морковь, яйцо, лук, майонез</t>
         </is>
       </c>
+      <c r="F26" t="n">
+        <v>390</v>
+      </c>
+      <c r="G26" t="n">
+        <v>12</v>
+      </c>
+      <c r="H26" t="n">
+        <v>30</v>
+      </c>
+      <c r="I26" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1089,6 +1413,18 @@
           <t>product_1778795345545_73d78bbf0710.webp</t>
         </is>
       </c>
+      <c r="F27" t="n">
+        <v>330</v>
+      </c>
+      <c r="G27" t="n">
+        <v>20</v>
+      </c>
+      <c r="H27" t="n">
+        <v>18</v>
+      </c>
+      <c r="I27" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1114,6 +1450,18 @@
           <t>product_1778795435326_b96ace57e65b.webp</t>
         </is>
       </c>
+      <c r="F28" t="n">
+        <v>398</v>
+      </c>
+      <c r="G28" t="n">
+        <v>22</v>
+      </c>
+      <c r="H28" t="n">
+        <v>22</v>
+      </c>
+      <c r="I28" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1139,6 +1487,18 @@
           <t>product_1778795530385_0b8b8a2770b5.webp</t>
         </is>
       </c>
+      <c r="F29" t="n">
+        <v>316</v>
+      </c>
+      <c r="G29" t="n">
+        <v>16</v>
+      </c>
+      <c r="H29" t="n">
+        <v>12</v>
+      </c>
+      <c r="I29" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1164,6 +1524,18 @@
           <t>product_1778795636944_921991e0acc9.webp</t>
         </is>
       </c>
+      <c r="F30" t="n">
+        <v>416</v>
+      </c>
+      <c r="G30" t="n">
+        <v>20</v>
+      </c>
+      <c r="H30" t="n">
+        <v>16</v>
+      </c>
+      <c r="I30" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1189,6 +1561,18 @@
           <t>product_1778795726841_c1c945379e9a.webp</t>
         </is>
       </c>
+      <c r="F31" t="n">
+        <v>474</v>
+      </c>
+      <c r="G31" t="n">
+        <v>22</v>
+      </c>
+      <c r="H31" t="n">
+        <v>18</v>
+      </c>
+      <c r="I31" t="n">
+        <v>56</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1214,6 +1598,18 @@
           <t>product_1778796375422_b37c4e5a30c7.webp</t>
         </is>
       </c>
+      <c r="F32" t="n">
+        <v>276</v>
+      </c>
+      <c r="G32" t="n">
+        <v>16</v>
+      </c>
+      <c r="H32" t="n">
+        <v>20</v>
+      </c>
+      <c r="I32" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1239,6 +1635,18 @@
           <t>product_1780238678005_f62d7bd82599.webp</t>
         </is>
       </c>
+      <c r="F33" t="n">
+        <v>244</v>
+      </c>
+      <c r="G33" t="n">
+        <v>14</v>
+      </c>
+      <c r="H33" t="n">
+        <v>12</v>
+      </c>
+      <c r="I33" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1264,6 +1672,18 @@
           <t>product_1780238714370_b1471c6a40f9.jpg</t>
         </is>
       </c>
+      <c r="F34" t="n">
+        <v>304</v>
+      </c>
+      <c r="G34" t="n">
+        <v>16</v>
+      </c>
+      <c r="H34" t="n">
+        <v>16</v>
+      </c>
+      <c r="I34" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1289,6 +1709,18 @@
           <t>product_1780238826173_8230cf602251.webp</t>
         </is>
       </c>
+      <c r="F35" t="n">
+        <v>240</v>
+      </c>
+      <c r="G35" t="n">
+        <v>18</v>
+      </c>
+      <c r="H35" t="n">
+        <v>8</v>
+      </c>
+      <c r="I35" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1314,6 +1746,18 @@
           <t>product_1780238857800_f06c7dc0b589.webp</t>
         </is>
       </c>
+      <c r="F36" t="n">
+        <v>252</v>
+      </c>
+      <c r="G36" t="n">
+        <v>5</v>
+      </c>
+      <c r="H36" t="n">
+        <v>16</v>
+      </c>
+      <c r="I36" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1339,6 +1783,18 @@
           <t>product_1778796756708_cee89af384a1.webp</t>
         </is>
       </c>
+      <c r="F37" t="n">
+        <v>742</v>
+      </c>
+      <c r="G37" t="n">
+        <v>42</v>
+      </c>
+      <c r="H37" t="n">
+        <v>46</v>
+      </c>
+      <c r="I37" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1364,6 +1820,18 @@
           <t>product_1778796858951_55a03ae15ae4.webp</t>
         </is>
       </c>
+      <c r="F38" t="n">
+        <v>594</v>
+      </c>
+      <c r="G38" t="n">
+        <v>34</v>
+      </c>
+      <c r="H38" t="n">
+        <v>34</v>
+      </c>
+      <c r="I38" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1389,6 +1857,18 @@
           <t>product_1778796953566_f1f584d21ee5.webp</t>
         </is>
       </c>
+      <c r="F39" t="n">
+        <v>676</v>
+      </c>
+      <c r="G39" t="n">
+        <v>32</v>
+      </c>
+      <c r="H39" t="n">
+        <v>44</v>
+      </c>
+      <c r="I39" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1414,6 +1894,18 @@
           <t>product_1778797048199_ff0eb9d5d61d.jpg</t>
         </is>
       </c>
+      <c r="F40" t="n">
+        <v>608</v>
+      </c>
+      <c r="G40" t="n">
+        <v>32</v>
+      </c>
+      <c r="H40" t="n">
+        <v>40</v>
+      </c>
+      <c r="I40" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1439,6 +1931,18 @@
           <t>product_1778797124342_7d187a0787a2.jpg</t>
         </is>
       </c>
+      <c r="F41" t="n">
+        <v>690</v>
+      </c>
+      <c r="G41" t="n">
+        <v>30</v>
+      </c>
+      <c r="H41" t="n">
+        <v>50</v>
+      </c>
+      <c r="I41" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1464,6 +1968,18 @@
           <t>product_1778797210571_ab095ba4b2be.webp</t>
         </is>
       </c>
+      <c r="F42" t="n">
+        <v>552</v>
+      </c>
+      <c r="G42" t="n">
+        <v>24</v>
+      </c>
+      <c r="H42" t="n">
+        <v>24</v>
+      </c>
+      <c r="I42" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1489,6 +2005,18 @@
           <t>product_1778797279444_a5c2c31b7a63.webp</t>
         </is>
       </c>
+      <c r="F43" t="n">
+        <v>392</v>
+      </c>
+      <c r="G43" t="n">
+        <v>36</v>
+      </c>
+      <c r="H43" t="n">
+        <v>24</v>
+      </c>
+      <c r="I43" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1514,6 +2042,18 @@
           <t>product_1778797647038_85d2cbc7c9ac.webp</t>
         </is>
       </c>
+      <c r="F44" t="n">
+        <v>526</v>
+      </c>
+      <c r="G44" t="n">
+        <v>30</v>
+      </c>
+      <c r="H44" t="n">
+        <v>30</v>
+      </c>
+      <c r="I44" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1539,6 +2079,18 @@
           <t>product_1778797743778_25c8788cb99a.jpg</t>
         </is>
       </c>
+      <c r="F45" t="n">
+        <v>428</v>
+      </c>
+      <c r="G45" t="n">
+        <v>32</v>
+      </c>
+      <c r="H45" t="n">
+        <v>20</v>
+      </c>
+      <c r="I45" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1564,6 +2116,18 @@
           <t>product_1778797816035_d448f234819f.jpg</t>
         </is>
       </c>
+      <c r="F46" t="n">
+        <v>464</v>
+      </c>
+      <c r="G46" t="n">
+        <v>32</v>
+      </c>
+      <c r="H46" t="n">
+        <v>24</v>
+      </c>
+      <c r="I46" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1589,6 +2153,18 @@
           <t>product_1778797887824_5b940e61fb3d.webp</t>
         </is>
       </c>
+      <c r="F47" t="n">
+        <v>338</v>
+      </c>
+      <c r="G47" t="n">
+        <v>20</v>
+      </c>
+      <c r="H47" t="n">
+        <v>18</v>
+      </c>
+      <c r="I47" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1614,6 +2190,18 @@
           <t>product_1778797994467_3bf589ef42a5.webp</t>
         </is>
       </c>
+      <c r="F48" t="n">
+        <v>358</v>
+      </c>
+      <c r="G48" t="n">
+        <v>20</v>
+      </c>
+      <c r="H48" t="n">
+        <v>22</v>
+      </c>
+      <c r="I48" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1639,6 +2227,18 @@
           <t>product_1778798067135_9a9da4780255.jpg</t>
         </is>
       </c>
+      <c r="F49" t="n">
+        <v>516</v>
+      </c>
+      <c r="G49" t="n">
+        <v>14</v>
+      </c>
+      <c r="H49" t="n">
+        <v>28</v>
+      </c>
+      <c r="I49" t="n">
+        <v>52</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1664,6 +2264,18 @@
           <t>product_1780238904095_1234fcbdc2ed.jpg</t>
         </is>
       </c>
+      <c r="F50" t="n">
+        <v>374</v>
+      </c>
+      <c r="G50" t="n">
+        <v>32</v>
+      </c>
+      <c r="H50" t="n">
+        <v>22</v>
+      </c>
+      <c r="I50" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1689,6 +2301,18 @@
           <t>product_1780239308621_19ee60811ff2.jpg</t>
         </is>
       </c>
+      <c r="F51" t="n">
+        <v>410</v>
+      </c>
+      <c r="G51" t="n">
+        <v>32</v>
+      </c>
+      <c r="H51" t="n">
+        <v>26</v>
+      </c>
+      <c r="I51" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1714,6 +2338,18 @@
           <t>product_1778798759460_603595e10e1f.webp</t>
         </is>
       </c>
+      <c r="F52" t="n">
+        <v>462</v>
+      </c>
+      <c r="G52" t="n">
+        <v>26</v>
+      </c>
+      <c r="H52" t="n">
+        <v>22</v>
+      </c>
+      <c r="I52" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1739,6 +2375,18 @@
           <t>product_1778798868157_7b72e012c1c3.webp</t>
         </is>
       </c>
+      <c r="F53" t="n">
+        <v>516</v>
+      </c>
+      <c r="G53" t="n">
+        <v>26</v>
+      </c>
+      <c r="H53" t="n">
+        <v>28</v>
+      </c>
+      <c r="I53" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1764,6 +2412,18 @@
           <t>product_1778798933888_7a3766645b15.webp</t>
         </is>
       </c>
+      <c r="F54" t="n">
+        <v>398</v>
+      </c>
+      <c r="G54" t="n">
+        <v>26</v>
+      </c>
+      <c r="H54" t="n">
+        <v>30</v>
+      </c>
+      <c r="I54" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1789,6 +2449,18 @@
           <t>product_1780607616870_58c9dc627c88.jpg</t>
         </is>
       </c>
+      <c r="F55" t="n">
+        <v>350</v>
+      </c>
+      <c r="G55" t="n">
+        <v>26</v>
+      </c>
+      <c r="H55" t="n">
+        <v>22</v>
+      </c>
+      <c r="I55" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1814,6 +2486,18 @@
           <t>product_1778799595056_9c4fda53cd46.webp</t>
         </is>
       </c>
+      <c r="F56" t="n">
+        <v>682</v>
+      </c>
+      <c r="G56" t="n">
+        <v>24</v>
+      </c>
+      <c r="H56" t="n">
+        <v>34</v>
+      </c>
+      <c r="I56" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1834,6 +2518,18 @@
           <t>Рис девзира, баранина, жёлтая морковь, лук, перепелиные яйца, казы, зира — на компанию</t>
         </is>
       </c>
+      <c r="F57" t="n">
+        <v>4460</v>
+      </c>
+      <c r="G57" t="n">
+        <v>160</v>
+      </c>
+      <c r="H57" t="n">
+        <v>220</v>
+      </c>
+      <c r="I57" t="n">
+        <v>460</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1854,6 +2550,18 @@
           <t>Говядина, картофель, лук, сладкий перец, чеснок, кинза</t>
         </is>
       </c>
+      <c r="F58" t="n">
+        <v>508</v>
+      </c>
+      <c r="G58" t="n">
+        <v>30</v>
+      </c>
+      <c r="H58" t="n">
+        <v>28</v>
+      </c>
+      <c r="I58" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1874,6 +2582,18 @@
           <t>Баранина, картофель, лук, сладкий перец, чеснок, кинза</t>
         </is>
       </c>
+      <c r="F59" t="n">
+        <v>572</v>
+      </c>
+      <c r="G59" t="n">
+        <v>28</v>
+      </c>
+      <c r="H59" t="n">
+        <v>36</v>
+      </c>
+      <c r="I59" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1899,6 +2619,18 @@
           <t>product_1780491704604_3b98bd72a88b.jpg</t>
         </is>
       </c>
+      <c r="F60" t="n">
+        <v>974</v>
+      </c>
+      <c r="G60" t="n">
+        <v>80</v>
+      </c>
+      <c r="H60" t="n">
+        <v>70</v>
+      </c>
+      <c r="I60" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1924,6 +2656,18 @@
           <t>product_1778799876348_0e6569cc0d63.webp</t>
         </is>
       </c>
+      <c r="F61" t="n">
+        <v>604</v>
+      </c>
+      <c r="G61" t="n">
+        <v>32</v>
+      </c>
+      <c r="H61" t="n">
+        <v>52</v>
+      </c>
+      <c r="I61" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1949,6 +2693,18 @@
           <t>product_1780242816420_7819a02749f6.jpg</t>
         </is>
       </c>
+      <c r="F62" t="n">
+        <v>564</v>
+      </c>
+      <c r="G62" t="n">
+        <v>30</v>
+      </c>
+      <c r="H62" t="n">
+        <v>48</v>
+      </c>
+      <c r="I62" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1974,6 +2730,18 @@
           <t>product_1780491181656_9b738405d967.webp</t>
         </is>
       </c>
+      <c r="F63" t="n">
+        <v>574</v>
+      </c>
+      <c r="G63" t="n">
+        <v>28</v>
+      </c>
+      <c r="H63" t="n">
+        <v>50</v>
+      </c>
+      <c r="I63" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1999,6 +2767,18 @@
           <t>product_1778852188678_5422dac03bdc.jpg</t>
         </is>
       </c>
+      <c r="F64" t="n">
+        <v>604</v>
+      </c>
+      <c r="G64" t="n">
+        <v>32</v>
+      </c>
+      <c r="H64" t="n">
+        <v>52</v>
+      </c>
+      <c r="I64" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2024,6 +2804,18 @@
           <t>product_1778852250396_94d15f9b8d71.webp</t>
         </is>
       </c>
+      <c r="F65" t="n">
+        <v>480</v>
+      </c>
+      <c r="G65" t="n">
+        <v>36</v>
+      </c>
+      <c r="H65" t="n">
+        <v>36</v>
+      </c>
+      <c r="I65" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2049,6 +2841,18 @@
           <t>product_1778852331329_942f5bc0b74e.webp</t>
         </is>
       </c>
+      <c r="F66" t="n">
+        <v>532</v>
+      </c>
+      <c r="G66" t="n">
+        <v>30</v>
+      </c>
+      <c r="H66" t="n">
+        <v>44</v>
+      </c>
+      <c r="I66" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2074,6 +2878,18 @@
           <t>product_1780242845512_77e6369709d2.jpg</t>
         </is>
       </c>
+      <c r="F67" t="n">
+        <v>744</v>
+      </c>
+      <c r="G67" t="n">
+        <v>6</v>
+      </c>
+      <c r="H67" t="n">
+        <v>80</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2099,6 +2915,18 @@
           <t>product_1778852450555_b9f5b85014f2.webp</t>
         </is>
       </c>
+      <c r="F68" t="n">
+        <v>302</v>
+      </c>
+      <c r="G68" t="n">
+        <v>42</v>
+      </c>
+      <c r="H68" t="n">
+        <v>14</v>
+      </c>
+      <c r="I68" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2124,6 +2952,18 @@
           <t>product_1778852498934_3a761a6b5fcb.webp</t>
         </is>
       </c>
+      <c r="F69" t="n">
+        <v>450</v>
+      </c>
+      <c r="G69" t="n">
+        <v>32</v>
+      </c>
+      <c r="H69" t="n">
+        <v>34</v>
+      </c>
+      <c r="I69" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2149,6 +2989,18 @@
           <t>product_1778852552042_e7da38ab5883.jpg</t>
         </is>
       </c>
+      <c r="F70" t="n">
+        <v>354</v>
+      </c>
+      <c r="G70" t="n">
+        <v>36</v>
+      </c>
+      <c r="H70" t="n">
+        <v>22</v>
+      </c>
+      <c r="I70" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2174,6 +3026,18 @@
           <t>product_1778852633425_787ff9d6a01c.webp</t>
         </is>
       </c>
+      <c r="F71" t="n">
+        <v>260</v>
+      </c>
+      <c r="G71" t="n">
+        <v>44</v>
+      </c>
+      <c r="H71" t="n">
+        <v>8</v>
+      </c>
+      <c r="I71" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2199,6 +3063,18 @@
           <t>product_1778852690213_21a951e72358.jpg</t>
         </is>
       </c>
+      <c r="F72" t="n">
+        <v>448</v>
+      </c>
+      <c r="G72" t="n">
+        <v>36</v>
+      </c>
+      <c r="H72" t="n">
+        <v>32</v>
+      </c>
+      <c r="I72" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2224,6 +3100,18 @@
           <t>product_1778852744685_cc730acd808f.jpg</t>
         </is>
       </c>
+      <c r="F73" t="n">
+        <v>178</v>
+      </c>
+      <c r="G73" t="n">
+        <v>4</v>
+      </c>
+      <c r="H73" t="n">
+        <v>10</v>
+      </c>
+      <c r="I73" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2249,6 +3137,18 @@
           <t>product_1780242916609_b48bcc4b05ca.jpg</t>
         </is>
       </c>
+      <c r="F74" t="n">
+        <v>138</v>
+      </c>
+      <c r="G74" t="n">
+        <v>8</v>
+      </c>
+      <c r="H74" t="n">
+        <v>10</v>
+      </c>
+      <c r="I74" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2274,6 +3174,18 @@
           <t>product_1778498923384_6b8fc75732bf.webp</t>
         </is>
       </c>
+      <c r="F75" t="n">
+        <v>434</v>
+      </c>
+      <c r="G75" t="n">
+        <v>7</v>
+      </c>
+      <c r="H75" t="n">
+        <v>22</v>
+      </c>
+      <c r="I75" t="n">
+        <v>52</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2299,6 +3211,18 @@
           <t>product_1778499030379_6c37cad6c068.webp</t>
         </is>
       </c>
+      <c r="F76" t="n">
+        <v>458</v>
+      </c>
+      <c r="G76" t="n">
+        <v>6</v>
+      </c>
+      <c r="H76" t="n">
+        <v>26</v>
+      </c>
+      <c r="I76" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2324,6 +3248,18 @@
           <t>product_1778499065579_27c61062830b.webp</t>
         </is>
       </c>
+      <c r="F77" t="n">
+        <v>514</v>
+      </c>
+      <c r="G77" t="n">
+        <v>9</v>
+      </c>
+      <c r="H77" t="n">
+        <v>30</v>
+      </c>
+      <c r="I77" t="n">
+        <v>52</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2349,6 +3285,18 @@
           <t>product_1778499114452_dfc463073c93.webp</t>
         </is>
       </c>
+      <c r="F78" t="n">
+        <v>446</v>
+      </c>
+      <c r="G78" t="n">
+        <v>6</v>
+      </c>
+      <c r="H78" t="n">
+        <v>22</v>
+      </c>
+      <c r="I78" t="n">
+        <v>56</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2374,6 +3322,18 @@
           <t>product_1780239954136_95c52443b759.webp</t>
         </is>
       </c>
+      <c r="F79" t="n">
+        <v>474</v>
+      </c>
+      <c r="G79" t="n">
+        <v>6</v>
+      </c>
+      <c r="H79" t="n">
+        <v>26</v>
+      </c>
+      <c r="I79" t="n">
+        <v>54</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2399,6 +3359,18 @@
           <t>product_1780491999204_54032d908297.webp</t>
         </is>
       </c>
+      <c r="F80" t="n">
+        <v>286</v>
+      </c>
+      <c r="G80" t="n">
+        <v>4</v>
+      </c>
+      <c r="H80" t="n">
+        <v>14</v>
+      </c>
+      <c r="I80" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2424,6 +3396,18 @@
           <t>product_1780492178966_e7da85c24a95.jpg</t>
         </is>
       </c>
+      <c r="F81" t="n">
+        <v>402</v>
+      </c>
+      <c r="G81" t="n">
+        <v>5</v>
+      </c>
+      <c r="H81" t="n">
+        <v>22</v>
+      </c>
+      <c r="I81" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2449,6 +3433,18 @@
           <t>product_1780240167810_b0ca510e7209.webp</t>
         </is>
       </c>
+      <c r="F82" t="n">
+        <v>180</v>
+      </c>
+      <c r="G82" t="n">
+        <v>3</v>
+      </c>
+      <c r="H82" t="n">
+        <v>8</v>
+      </c>
+      <c r="I82" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2474,6 +3470,18 @@
           <t>product_1780240206109_e3ee61d5df13.webp</t>
         </is>
       </c>
+      <c r="F83" t="n">
+        <v>228</v>
+      </c>
+      <c r="G83" t="n">
+        <v>4</v>
+      </c>
+      <c r="H83" t="n">
+        <v>4</v>
+      </c>
+      <c r="I83" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2499,6 +3507,18 @@
           <t>product_1780240237235_dbcaee760521.webp</t>
         </is>
       </c>
+      <c r="F84" t="n">
+        <v>197</v>
+      </c>
+      <c r="G84" t="n">
+        <v>6</v>
+      </c>
+      <c r="H84" t="n">
+        <v>5</v>
+      </c>
+      <c r="I84" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2524,6 +3544,18 @@
           <t>product_1780492357919_bb1fb7d51ef7.webp</t>
         </is>
       </c>
+      <c r="F85" t="n">
+        <v>237</v>
+      </c>
+      <c r="G85" t="n">
+        <v>6</v>
+      </c>
+      <c r="H85" t="n">
+        <v>5</v>
+      </c>
+      <c r="I85" t="n">
+        <v>42</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2549,6 +3581,18 @@
           <t>product_1780240397657_662e26897931.webp</t>
         </is>
       </c>
+      <c r="F86" t="n">
+        <v>510</v>
+      </c>
+      <c r="G86" t="n">
+        <v>16</v>
+      </c>
+      <c r="H86" t="n">
+        <v>6</v>
+      </c>
+      <c r="I86" t="n">
+        <v>98</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2574,6 +3618,18 @@
           <t>product_1780492845588_efab13909377.webp</t>
         </is>
       </c>
+      <c r="F87" t="n">
+        <v>638</v>
+      </c>
+      <c r="G87" t="n">
+        <v>12</v>
+      </c>
+      <c r="H87" t="n">
+        <v>30</v>
+      </c>
+      <c r="I87" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2599,6 +3655,18 @@
           <t>product_1780493182684_a63698c3b017.webp</t>
         </is>
       </c>
+      <c r="F88" t="n">
+        <v>138</v>
+      </c>
+      <c r="G88" t="n">
+        <v>1</v>
+      </c>
+      <c r="H88" t="n">
+        <v>14</v>
+      </c>
+      <c r="I88" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2624,6 +3692,18 @@
           <t>product_1780493296737_814038eb5bdb.jpg</t>
         </is>
       </c>
+      <c r="F89" t="n">
+        <v>37</v>
+      </c>
+      <c r="G89" t="n">
+        <v>1</v>
+      </c>
+      <c r="H89" t="n">
+        <v>1</v>
+      </c>
+      <c r="I89" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2649,6 +3729,18 @@
           <t>product_1780493354418_3a4a4d6bac45.jpg</t>
         </is>
       </c>
+      <c r="F90" t="n">
+        <v>38</v>
+      </c>
+      <c r="G90" t="n">
+        <v>1</v>
+      </c>
+      <c r="H90" t="n">
+        <v>2</v>
+      </c>
+      <c r="I90" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2674,6 +3766,18 @@
           <t>product_1780493340076_f52cdd8bc0f5.webp</t>
         </is>
       </c>
+      <c r="F91" t="n">
+        <v>29</v>
+      </c>
+      <c r="G91" t="n">
+        <v>1</v>
+      </c>
+      <c r="H91" t="n">
+        <v>1</v>
+      </c>
+      <c r="I91" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2699,6 +3803,18 @@
           <t>product_1780493368934_145f9dc334b0.webp</t>
         </is>
       </c>
+      <c r="F92" t="n">
+        <v>102</v>
+      </c>
+      <c r="G92" t="n">
+        <v>1</v>
+      </c>
+      <c r="H92" t="n">
+        <v>10</v>
+      </c>
+      <c r="I92" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2724,6 +3840,18 @@
           <t>product_1780493384080_d51613e3f6d2.jpg</t>
         </is>
       </c>
+      <c r="F93" t="n">
+        <v>52</v>
+      </c>
+      <c r="G93" t="n">
+        <v>1</v>
+      </c>
+      <c r="H93" t="n">
+        <v>0</v>
+      </c>
+      <c r="I93" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2749,6 +3877,18 @@
           <t>product_1780608795851_902a4ff3f798.webp</t>
         </is>
       </c>
+      <c r="F94" t="n">
+        <v>96</v>
+      </c>
+      <c r="G94" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" t="n">
+        <v>0</v>
+      </c>
+      <c r="I94" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2774,6 +3914,18 @@
           <t>product_1780608857167_49eb4f5abf58.webp</t>
         </is>
       </c>
+      <c r="F95" t="n">
+        <v>0</v>
+      </c>
+      <c r="G95" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" t="n">
+        <v>0</v>
+      </c>
+      <c r="I95" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2799,6 +3951,18 @@
           <t>product_1780608990754_5f403ccaa97c.webp</t>
         </is>
       </c>
+      <c r="F96" t="n">
+        <v>0</v>
+      </c>
+      <c r="G96" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" t="n">
+        <v>0</v>
+      </c>
+      <c r="I96" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2824,6 +3988,18 @@
           <t>product_1780609109425_7fc26e9c2550.webp</t>
         </is>
       </c>
+      <c r="F97" t="n">
+        <v>0</v>
+      </c>
+      <c r="G97" t="n">
+        <v>0</v>
+      </c>
+      <c r="H97" t="n">
+        <v>0</v>
+      </c>
+      <c r="I97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2849,6 +4025,18 @@
           <t>product_1780609226786_1564810ae109.webp</t>
         </is>
       </c>
+      <c r="F98" t="n">
+        <v>0</v>
+      </c>
+      <c r="G98" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" t="n">
+        <v>0</v>
+      </c>
+      <c r="I98" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2874,6 +4062,18 @@
           <t>product_1780609322092_c94204cd75f4.webp</t>
         </is>
       </c>
+      <c r="F99" t="n">
+        <v>0</v>
+      </c>
+      <c r="G99" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" t="n">
+        <v>0</v>
+      </c>
+      <c r="I99" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2899,6 +4099,18 @@
           <t>product_1780609372516_a5d0a7d31b44.webp</t>
         </is>
       </c>
+      <c r="F100" t="n">
+        <v>0</v>
+      </c>
+      <c r="G100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H100" t="n">
+        <v>0</v>
+      </c>
+      <c r="I100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2924,6 +4136,18 @@
           <t>product_1780609704522_c3b5837c0f9e.jpg</t>
         </is>
       </c>
+      <c r="F101" t="n">
+        <v>0</v>
+      </c>
+      <c r="G101" t="n">
+        <v>0</v>
+      </c>
+      <c r="H101" t="n">
+        <v>0</v>
+      </c>
+      <c r="I101" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2949,6 +4173,18 @@
           <t>product_1780609820023_ba01c1ac2228.webp</t>
         </is>
       </c>
+      <c r="F102" t="n">
+        <v>120</v>
+      </c>
+      <c r="G102" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" t="n">
+        <v>0</v>
+      </c>
+      <c r="I102" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2974,6 +4210,18 @@
           <t>product_1780609882480_9efe401c2312.webp</t>
         </is>
       </c>
+      <c r="F103" t="n">
+        <v>128</v>
+      </c>
+      <c r="G103" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" t="n">
+        <v>0</v>
+      </c>
+      <c r="I103" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2999,6 +4247,18 @@
           <t>product_1780609939629_a425c39a83bb.webp</t>
         </is>
       </c>
+      <c r="F104" t="n">
+        <v>104</v>
+      </c>
+      <c r="G104" t="n">
+        <v>0</v>
+      </c>
+      <c r="H104" t="n">
+        <v>0</v>
+      </c>
+      <c r="I104" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -3024,6 +4284,18 @@
           <t>product_1780610005205_a2df7641f81b.webp</t>
         </is>
       </c>
+      <c r="F105" t="n">
+        <v>104</v>
+      </c>
+      <c r="G105" t="n">
+        <v>0</v>
+      </c>
+      <c r="H105" t="n">
+        <v>0</v>
+      </c>
+      <c r="I105" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -3049,6 +4321,18 @@
           <t>product_1780610052293_0792274c1599.webp</t>
         </is>
       </c>
+      <c r="F106" t="n">
+        <v>80</v>
+      </c>
+      <c r="G106" t="n">
+        <v>0</v>
+      </c>
+      <c r="H106" t="n">
+        <v>0</v>
+      </c>
+      <c r="I106" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -3074,6 +4358,18 @@
           <t>product_1780610096481_5e0f506a071f.webp</t>
         </is>
       </c>
+      <c r="F107" t="n">
+        <v>64</v>
+      </c>
+      <c r="G107" t="n">
+        <v>0</v>
+      </c>
+      <c r="H107" t="n">
+        <v>0</v>
+      </c>
+      <c r="I107" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3099,6 +4395,18 @@
           <t>product_1780610296823_29d76a0fb113.webp</t>
         </is>
       </c>
+      <c r="F108" t="n">
+        <v>104</v>
+      </c>
+      <c r="G108" t="n">
+        <v>0</v>
+      </c>
+      <c r="H108" t="n">
+        <v>0</v>
+      </c>
+      <c r="I108" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -3124,6 +4432,18 @@
           <t>product_1780610402868_00fc5f95b509.webp</t>
         </is>
       </c>
+      <c r="F109" t="n">
+        <v>112</v>
+      </c>
+      <c r="G109" t="n">
+        <v>0</v>
+      </c>
+      <c r="H109" t="n">
+        <v>0</v>
+      </c>
+      <c r="I109" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -3149,6 +4469,18 @@
           <t>product_1780610557472_aa235338f77a.webp</t>
         </is>
       </c>
+      <c r="F110" t="n">
+        <v>88</v>
+      </c>
+      <c r="G110" t="n">
+        <v>0</v>
+      </c>
+      <c r="H110" t="n">
+        <v>0</v>
+      </c>
+      <c r="I110" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3174,6 +4506,18 @@
           <t>product_1780610569393_43d760e6c097.webp</t>
         </is>
       </c>
+      <c r="F111" t="n">
+        <v>444</v>
+      </c>
+      <c r="G111" t="n">
+        <v>1</v>
+      </c>
+      <c r="H111" t="n">
+        <v>0</v>
+      </c>
+      <c r="I111" t="n">
+        <v>110</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3199,6 +4543,18 @@
           <t>product_1780610642670_8a53254e7afa.webp</t>
         </is>
       </c>
+      <c r="F112" t="n">
+        <v>460</v>
+      </c>
+      <c r="G112" t="n">
+        <v>5</v>
+      </c>
+      <c r="H112" t="n">
+        <v>0</v>
+      </c>
+      <c r="I112" t="n">
+        <v>110</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3224,6 +4580,18 @@
           <t>product_1780610748304_4e685c4c4183.webp</t>
         </is>
       </c>
+      <c r="F113" t="n">
+        <v>0</v>
+      </c>
+      <c r="G113" t="n">
+        <v>0</v>
+      </c>
+      <c r="H113" t="n">
+        <v>0</v>
+      </c>
+      <c r="I113" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3249,6 +4617,18 @@
           <t>product_1780610782635_77a78b588901.webp</t>
         </is>
       </c>
+      <c r="F114" t="n">
+        <v>0</v>
+      </c>
+      <c r="G114" t="n">
+        <v>0</v>
+      </c>
+      <c r="H114" t="n">
+        <v>0</v>
+      </c>
+      <c r="I114" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3274,6 +4654,18 @@
           <t>product_1780610794035_27bbadc3e91a.webp</t>
         </is>
       </c>
+      <c r="F115" t="n">
+        <v>0</v>
+      </c>
+      <c r="G115" t="n">
+        <v>0</v>
+      </c>
+      <c r="H115" t="n">
+        <v>0</v>
+      </c>
+      <c r="I115" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -3299,6 +4691,18 @@
           <t>product_1780610839722_3b4c572f7170.webp</t>
         </is>
       </c>
+      <c r="F116" t="n">
+        <v>128</v>
+      </c>
+      <c r="G116" t="n">
+        <v>0</v>
+      </c>
+      <c r="H116" t="n">
+        <v>0</v>
+      </c>
+      <c r="I116" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -3324,6 +4728,18 @@
           <t>product_1780610850313_9463c44ad93c.webp</t>
         </is>
       </c>
+      <c r="F117" t="n">
+        <v>320</v>
+      </c>
+      <c r="G117" t="n">
+        <v>0</v>
+      </c>
+      <c r="H117" t="n">
+        <v>0</v>
+      </c>
+      <c r="I117" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3349,6 +4765,18 @@
           <t>product_1780610895968_b28342fd0dd5.webp</t>
         </is>
       </c>
+      <c r="F118" t="n">
+        <v>152</v>
+      </c>
+      <c r="G118" t="n">
+        <v>0</v>
+      </c>
+      <c r="H118" t="n">
+        <v>0</v>
+      </c>
+      <c r="I118" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3374,6 +4802,18 @@
           <t>product_1780610905578_17f7b9177aae.webp</t>
         </is>
       </c>
+      <c r="F119" t="n">
+        <v>384</v>
+      </c>
+      <c r="G119" t="n">
+        <v>1</v>
+      </c>
+      <c r="H119" t="n">
+        <v>0</v>
+      </c>
+      <c r="I119" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3399,6 +4839,18 @@
           <t>product_1780610971256_bc03ddcf4ccd.webp</t>
         </is>
       </c>
+      <c r="F120" t="n">
+        <v>172</v>
+      </c>
+      <c r="G120" t="n">
+        <v>1</v>
+      </c>
+      <c r="H120" t="n">
+        <v>0</v>
+      </c>
+      <c r="I120" t="n">
+        <v>42</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -3424,6 +4876,18 @@
           <t>product_1780610979571_76d3d8edc42d.webp</t>
         </is>
       </c>
+      <c r="F121" t="n">
+        <v>428</v>
+      </c>
+      <c r="G121" t="n">
+        <v>2</v>
+      </c>
+      <c r="H121" t="n">
+        <v>0</v>
+      </c>
+      <c r="I121" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -3449,6 +4913,18 @@
           <t>product_1780611125871_7a67b3917609.webp</t>
         </is>
       </c>
+      <c r="F122" t="n">
+        <v>152</v>
+      </c>
+      <c r="G122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H122" t="n">
+        <v>0</v>
+      </c>
+      <c r="I122" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3474,6 +4950,18 @@
           <t>product_1780611138149_cbef850291cf.webp</t>
         </is>
       </c>
+      <c r="F123" t="n">
+        <v>384</v>
+      </c>
+      <c r="G123" t="n">
+        <v>1</v>
+      </c>
+      <c r="H123" t="n">
+        <v>0</v>
+      </c>
+      <c r="I123" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -3499,6 +4987,18 @@
           <t>product_1780611190246_e87a9a9447f1.webp</t>
         </is>
       </c>
+      <c r="F124" t="n">
+        <v>424</v>
+      </c>
+      <c r="G124" t="n">
+        <v>0</v>
+      </c>
+      <c r="H124" t="n">
+        <v>0</v>
+      </c>
+      <c r="I124" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -3524,6 +5024,18 @@
           <t>product_1780611200868_b35d6092fd27.webp</t>
         </is>
       </c>
+      <c r="F125" t="n">
+        <v>636</v>
+      </c>
+      <c r="G125" t="n">
+        <v>0</v>
+      </c>
+      <c r="H125" t="n">
+        <v>0</v>
+      </c>
+      <c r="I125" t="n">
+        <v>159</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -3549,6 +5061,18 @@
           <t>product_1780611249563_9d8a2bc7a43c.webp</t>
         </is>
       </c>
+      <c r="F126" t="n">
+        <v>220</v>
+      </c>
+      <c r="G126" t="n">
+        <v>0</v>
+      </c>
+      <c r="H126" t="n">
+        <v>0</v>
+      </c>
+      <c r="I126" t="n">
+        <v>55</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -3574,6 +5098,18 @@
           <t>product_1780611310927_65bcc56ed969.webp</t>
         </is>
       </c>
+      <c r="F127" t="n">
+        <v>200</v>
+      </c>
+      <c r="G127" t="n">
+        <v>0</v>
+      </c>
+      <c r="H127" t="n">
+        <v>0</v>
+      </c>
+      <c r="I127" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -3599,6 +5135,18 @@
           <t>product_1780611352464_8303415a5ba2.webp</t>
         </is>
       </c>
+      <c r="F128" t="n">
+        <v>228</v>
+      </c>
+      <c r="G128" t="n">
+        <v>0</v>
+      </c>
+      <c r="H128" t="n">
+        <v>0</v>
+      </c>
+      <c r="I128" t="n">
+        <v>57</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -3624,6 +5172,18 @@
           <t>product_1780611446247_0ea8863b3a53.webp</t>
         </is>
       </c>
+      <c r="F129" t="n">
+        <v>128</v>
+      </c>
+      <c r="G129" t="n">
+        <v>0</v>
+      </c>
+      <c r="H129" t="n">
+        <v>0</v>
+      </c>
+      <c r="I129" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -3644,6 +5204,18 @@
           <t>Газированный напиток</t>
         </is>
       </c>
+      <c r="F130" t="n">
+        <v>212</v>
+      </c>
+      <c r="G130" t="n">
+        <v>0</v>
+      </c>
+      <c r="H130" t="n">
+        <v>0</v>
+      </c>
+      <c r="I130" t="n">
+        <v>53</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -3664,6 +5236,18 @@
           <t>Газированный напиток</t>
         </is>
       </c>
+      <c r="F131" t="n">
+        <v>424</v>
+      </c>
+      <c r="G131" t="n">
+        <v>0</v>
+      </c>
+      <c r="H131" t="n">
+        <v>0</v>
+      </c>
+      <c r="I131" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -3683,6 +5267,18 @@
         <is>
           <t>Газированный напиток</t>
         </is>
+      </c>
+      <c r="F132" t="n">
+        <v>848</v>
+      </c>
+      <c r="G132" t="n">
+        <v>0</v>
+      </c>
+      <c r="H132" t="n">
+        <v>0</v>
+      </c>
+      <c r="I132" t="n">
+        <v>212</v>
       </c>
     </row>
   </sheetData>

</xml_diff>